<commit_message>
feat(power): incorporate Phoenix Contact TRIO 20A (2903151) from JW Tech quotation QJP-260901724-R0 into panel power design
</commit_message>
<xml_diff>
--- a/03_IO_Lists_and_Schedules/Panel_Power_Supply_Calculation_Report.xlsx
+++ b/03_IO_Lists_and_Schedules/Panel_Power_Supply_Calculation_Report.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24VDC_Field_Load_Details" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AC_Mains_and_UPS_Sizing" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power_Equipment_BOM" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIO_Quotation_Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +109,12 @@
         <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -135,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -211,6 +218,17 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5073,4 +5091,1034 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="75" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PHOENIX CONTACT TRIO POWER (2903151) SIZING &amp; VERIFICATION --- JW TECH QUOTATION REF: QJP-260901724-R0</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>1. PROCUREMENT &amp; COMMERCIAL METADATA (QUOTATION QJP-260901724-R0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Quotation Number</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>QJP-260901724-R0</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n"/>
+      <c r="D4" s="20" t="n"/>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>Supplier / Vendor</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>JW TECH., LTD. (เลขที่ 226 ซอยศูนย์การค้าแฮปปี้แลนด์ 1 บางกะปิ กรุงเทพฯ)</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="n"/>
+      <c r="H4" s="20" t="n"/>
+      <c r="I4" s="20" t="n"/>
+      <c r="J4" s="20" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Quotation Date</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>11 กันยายน 2026 (11 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Vendor Contact</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>นางสาวจิรัชยา โพธิ์งาม (Tel: +66863101172, nidda@jwtech.co.th)</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="n"/>
+      <c r="H5" s="20" t="n"/>
+      <c r="I5" s="20" t="n"/>
+      <c r="J5" s="20" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Buyer / Client</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>บริษัท อีโคแมกซ์ เอ็นจิเนียริ่ง ซัพพลายแอนด์ เซอร์วิส จำกัด</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Attention</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Khun Surachet Jumpit (Tel: 089-8926578, info.ecomax3@gmail.com)</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="n"/>
+      <c r="H6" s="20" t="n"/>
+      <c r="I6" s="20" t="n"/>
+      <c r="J6" s="20" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Item Description</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Power supply unit, primary-switched, 1-phase AC, 24VDC, 20A</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n"/>
+      <c r="D7" s="20" t="n"/>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Part Number / Model</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2903151 --- TRIO-PS-2G/1AC/24DC/20</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="20" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Quoted Quantity</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>5 EA (In Stock)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="20" t="n"/>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>Unit Price (THB)</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>7,260.00 THB / EA</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="I8" s="20" t="n"/>
+      <c r="J8" s="20" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Subtotal Amount</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>36,300.00 THB</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="20" t="n"/>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Grand Total (+7% VAT)</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>38,841.00 THB (Payment: Cash, Warranty: 1 Year)</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="n"/>
+      <c r="H9" s="20" t="n"/>
+      <c r="I9" s="20" t="n"/>
+      <c r="J9" s="20" t="n"/>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>2. TECHNICAL PARAMETERS OF PHOENIX CONTACT TRIO-PS-2G/1AC/24DC/20 (2903151)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Nominal AC Input Voltage</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>100 V AC ... 240 V AC (-15% / +10%)</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>Efficiency @ 230VAC</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>&gt; 93.0% (Typical)</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="n"/>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Heat Dissipation (Max)</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>36.0 W @ 20A full load</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="n"/>
+      <c r="J12" s="20" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>AC Input Voltage Range</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>85 V AC ... 264 V AC (45 ... 65 Hz)</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Power Factor (cos phi)</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>0.95 (Built-in active PFC)</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="n"/>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Inrush Current</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 15 A @ 230VAC (Cold Start)</t>
+        </is>
+      </c>
+      <c r="I13" s="20" t="n"/>
+      <c r="J13" s="20" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Nominal Output Voltage</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>24 V DC (Adjustable 24 ... 28 V DC)</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="n"/>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Push-in Conductor Size</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>0.2 ... 4 mm² (In), 0.2 ... 10 mm² (Out)</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="n"/>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Housing Dimensions</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>68 x 130 x 160 mm (W x H x D)</t>
+        </is>
+      </c>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="20" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Nominal Output Current</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>20.0 A continuous (-25°C ... +60°C)</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n"/>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Dynamic Boost (150%)</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>30.0 A for 5 seconds (heavy startup)</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="n"/>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Status Contact</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>DC OK Floating Relay (30V, 100mA)</t>
+        </is>
+      </c>
+      <c r="I15" s="20" t="n"/>
+      <c r="J15" s="20" t="n"/>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>3. SIZING &amp; LOADING ANALYSIS --- 5 QUOTED UNITS ALLOCATION OPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>OPTION A: DEDICATED PER-CHASSIS DC DOMAIN (1x 20A TRIO PSU Per ControlLogix Chassis C1 to C5) --- RECOMMENDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t>Unit #</t>
+        </is>
+      </c>
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>Target Chassis</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>Panel &amp; Location</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="inlineStr">
+        <is>
+          <t>24VDC Oper. Load (A)</t>
+        </is>
+      </c>
+      <c r="E19" s="36" t="inlineStr">
+        <is>
+          <t>Design Load +30% (A)</t>
+        </is>
+      </c>
+      <c r="F19" s="36" t="inlineStr">
+        <is>
+          <t>TRIO Rated (A)</t>
+        </is>
+      </c>
+      <c r="G19" s="36" t="inlineStr">
+        <is>
+          <t>TRIO Utilization (%)</t>
+        </is>
+      </c>
+      <c r="H19" s="36" t="inlineStr">
+        <is>
+          <t>Dynamic Boost (5s)</t>
+        </is>
+      </c>
+      <c r="I19" s="36" t="inlineStr">
+        <is>
+          <t>Thermal Loss (W)</t>
+        </is>
+      </c>
+      <c r="J19" s="36" t="inlineStr">
+        <is>
+          <t>Engineering Sizing Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Unit 1</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Chassis C1</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>CA1 (Main Control Room)</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>48.5%</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>30.0 A (150%)</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J20" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Optimal Load &lt;50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Unit 2</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Chassis C2</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>CA1 (Main Control Room)</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>72.8%</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>30.0 A (150%)</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="J21" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Safe Continuous &lt;75%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Unit 3</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Chassis C3</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>CA-RIO-1 (Spray Dryer 3F/7F)</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>14.79</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>74.0%</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>30.0 A (150%)</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="J22" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Safe Continuous &lt;75%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Unit 4</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Chassis C4</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>CA-RIO-2 (Spray Dryer 6F/8F)</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="F23" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>36.2%</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>30.0 A (150%)</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J23" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Generous Spare Headroom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Unit 5</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Chassis C5</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>CA-RIO-200 (Slurry Building 2F)</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="F24" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>36.6%</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>30.0 A (150%)</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="J24" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Generous Spare Headroom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>OPTION B: PANEL-LEVEL REDUNDANT BUS (2x 20A in CA1 + 1x 20A in each Remote Panel) --- ALTERNATIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>Unit Allocation</t>
+        </is>
+      </c>
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>Target Panel</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>Location &amp; Role</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>Total 24VDC Load (A)</t>
+        </is>
+      </c>
+      <c r="E27" s="36" t="inlineStr">
+        <is>
+          <t>Design Load +30% (A)</t>
+        </is>
+      </c>
+      <c r="F27" s="36" t="inlineStr">
+        <is>
+          <t>Bus Capacity (A)</t>
+        </is>
+      </c>
+      <c r="G27" s="36" t="inlineStr">
+        <is>
+          <t>Redundancy / Mode</t>
+        </is>
+      </c>
+      <c r="H27" s="36" t="inlineStr">
+        <is>
+          <t>Single PSU Load</t>
+        </is>
+      </c>
+      <c r="I27" s="36" t="inlineStr">
+        <is>
+          <t>Thermal Loss (W)</t>
+        </is>
+      </c>
+      <c r="J27" s="36" t="inlineStr">
+        <is>
+          <t>Engineering Sizing Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Units 1 &amp; 2 (2 EA)</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Panel CA1</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Main Control Room (C1 + C2)</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>35.88</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>2x 20A Parallel / Redundant</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>89.7% (Single) / 44.9% (Dual)</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="J28" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Sufficient Bus Capacity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Unit 3 (1 EA)</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Panel CA-RIO-1</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Spray Dryer 3F/7F (C3)</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>14.79</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Single Switched Mode</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>74.0% of nominal 20A</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="J29" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Safe Continuous &lt;75%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Unit 4 (1 EA)</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Panel CA-RIO-2</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Spray Dryer 6F/8F (C4)</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Single Switched Mode</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>36.2% of nominal 20A</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J30" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Optimal &lt;50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Unit 5 (1 EA)</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Panel CA-RIO-200</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Slurry Building 2F (C5)</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Single Switched Mode</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>36.6% of nominal 20A</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="J31" s="37" t="inlineStr">
+        <is>
+          <t>PASS (Optimal &lt;50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="34" t="inlineStr">
+        <is>
+          <t>4. SWITCHGEAR PROTECTION &amp; PLC SCADA INTEGRATION DESIGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>AC Mains Infeed Protection</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>Each TRIO 20A unit must be protected by an upstream 2-Pole Miniature Circuit Breaker rated 10A (or 6A), Characteristic C (e.g. Schneider Acti9 iC60N 2P 10A C). Inrush current is &lt;15A, well below the C-curve magnetic trip threshold (50-100A).</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="n"/>
+      <c r="D34" s="20" t="n"/>
+      <c r="E34" s="20" t="n"/>
+      <c r="F34" s="20" t="n"/>
+      <c r="G34" s="20" t="n"/>
+      <c r="H34" s="20" t="n"/>
+      <c r="I34" s="20" t="n"/>
+      <c r="J34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>DC Output Distribution</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Branch feeds from each 24VDC TRIO power supply should be segregated using multi-channel electronic circuit breakers (Phoenix Contact PTCB or C60H-DC) to ensure selective trip during field sensor/solenoid short circuits without collapsing the 24V bus.</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+      <c r="E35" s="20" t="n"/>
+      <c r="F35" s="20" t="n"/>
+      <c r="G35" s="20" t="n"/>
+      <c r="H35" s="20" t="n"/>
+      <c r="I35" s="20" t="n"/>
+      <c r="J35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>DC OK Contact Supervision</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>The integrated floating relay contact (terminals 13/14, 30V AC/DC, 100mA) on each TRIO unit shall be hardwired directly into a spare channel on the 1756-IB32 digital input card (e.g. Tag: 'PSU_HEALTHY_CHx').</t>
+        </is>
+      </c>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="20" t="n"/>
+      <c r="E36" s="20" t="n"/>
+      <c r="F36" s="20" t="n"/>
+      <c r="G36" s="20" t="n"/>
+      <c r="H36" s="20" t="n"/>
+      <c r="I36" s="20" t="n"/>
+      <c r="J36" s="20" t="n"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>SCADA Alarm Logic</t>
+        </is>
+      </c>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>FactoryTalk View SE will display a yellow banner alarm if 'PSU_HEALTHY' de-energizes, alerting operators to power supply derating, AC line loss, or output under-voltage (&lt;21.5V) prior to PLC brownout.</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="20" t="n"/>
+      <c r="E37" s="20" t="n"/>
+      <c r="F37" s="20" t="n"/>
+      <c r="G37" s="20" t="n"/>
+      <c r="H37" s="20" t="n"/>
+      <c r="I37" s="20" t="n"/>
+      <c r="J37" s="20" t="n"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>Push-in Terminal Cabling</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>AC Input: 2.5 mm² multi-strand copper (THW / H07V-K) with insulated ferrule. DC Output: 6.0 mm² or 10.0 mm² copper (Red/Black) to main 24VDC terminal blocks Px-TBDC(+) and Px-TBDC(-).</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="n"/>
+      <c r="D38" s="20" t="n"/>
+      <c r="E38" s="20" t="n"/>
+      <c r="F38" s="20" t="n"/>
+      <c r="G38" s="20" t="n"/>
+      <c r="H38" s="20" t="n"/>
+      <c r="I38" s="20" t="n"/>
+      <c r="J38" s="20" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="36">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F7:J7"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F8:J8"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="F9:J9"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="F4:J4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(power): recalculate power consumption with true analog channel counts, pneumatic solenoid duty ratings, and P+F IS barrier loads
</commit_message>
<xml_diff>
--- a/03_IO_Lists_and_Schedules/Panel_Power_Supply_Calculation_Report.xlsx
+++ b/03_IO_Lists_and_Schedules/Panel_Power_Supply_Calculation_Report.xlsx
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>27.6</v>
+        <v>14.1</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>35.88</v>
+        <v>18.33</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
@@ -720,11 +720,11 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>89.7%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1439</v>
+        <v>972.2</v>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
@@ -733,11 +733,11 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>3000 VA (48.0% load)</t>
+          <t>3000 VA (32.4% load)</t>
         </is>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1574</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="8">
@@ -757,10 +757,10 @@
         </is>
       </c>
       <c r="D8" s="11" t="n">
-        <v>11.38</v>
+        <v>6.28</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>14.79</v>
+        <v>8.16</v>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
@@ -769,11 +769,11 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>73.9%</t>
+          <t>40.8%</t>
         </is>
       </c>
       <c r="H8" s="11" t="n">
-        <v>790.9</v>
+        <v>610.9</v>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
@@ -782,11 +782,11 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>1500 VA (52.7% load)</t>
+          <t>1500 VA (40.7% load)</t>
         </is>
       </c>
       <c r="K8" s="11" t="n">
-        <v>699</v>
+        <v>495</v>
       </c>
     </row>
     <row r="9">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>5.57</v>
+        <v>4.48</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7.24</v>
+        <v>5.83</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
@@ -818,11 +818,11 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>565.8</v>
+        <v>527.5</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
@@ -831,11 +831,11 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>1500 VA (37.7% load)</t>
+          <t>1500 VA (35.2% load)</t>
         </is>
       </c>
       <c r="K9" s="7" t="n">
-        <v>416</v>
+        <v>372</v>
       </c>
     </row>
     <row r="10">
@@ -855,10 +855,10 @@
         </is>
       </c>
       <c r="D10" s="11" t="n">
-        <v>5.63</v>
+        <v>4.1</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>7.32</v>
+        <v>5.34</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -867,11 +867,11 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>73.2%</t>
+          <t>53.4%</t>
         </is>
       </c>
       <c r="H10" s="11" t="n">
-        <v>555.8</v>
+        <v>500.6</v>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
@@ -880,11 +880,11 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>1000 VA (55.6% load)</t>
+          <t>1000 VA (50.1% load)</t>
         </is>
       </c>
       <c r="K10" s="11" t="n">
-        <v>378</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11">
@@ -904,10 +904,10 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>15.46</v>
+        <v>10.11</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>20.1</v>
+        <v>13.14</v>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
@@ -916,11 +916,11 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>50.3%</t>
+          <t>32.9%</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1003.8</v>
+        <v>801.9</v>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
@@ -929,11 +929,11 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>2000 VA (50.2% load)</t>
+          <t>2000 VA (40.1% load)</t>
         </is>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1064</v>
+        <v>814</v>
       </c>
     </row>
     <row r="12">
@@ -953,10 +953,10 @@
         </is>
       </c>
       <c r="D12" s="11" t="n">
-        <v>4.24</v>
+        <v>6.24</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>5.51</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
@@ -965,11 +965,11 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>27.5%</t>
+          <t>40.5%</t>
         </is>
       </c>
       <c r="H12" s="11" t="n">
-        <v>526.5</v>
+        <v>580.5</v>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
@@ -978,11 +978,11 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>1500 VA (35.1% load)</t>
+          <t>1500 VA (38.7% load)</t>
         </is>
       </c>
       <c r="K12" s="11" t="n">
-        <v>378</v>
+        <v>415</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>69.88</v>
+        <v>45.31</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>90.84</v>
+        <v>58.9</v>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>4881.8</v>
+        <v>3993.6</v>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="K13" s="14" t="n">
-        <v>4509</v>
+        <v>3463</v>
       </c>
     </row>
     <row r="14"/>
@@ -3821,13 +3821,13 @@
         <v>1.18</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>1.44</v>
+        <v>0.55</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>15.84</v>
+        <v>4.4</v>
       </c>
       <c r="F4" s="21" t="n">
-        <v>2.02</v>
+        <v>0.84</v>
       </c>
       <c r="G4" s="21" t="n">
         <v>0</v>
@@ -3839,10 +3839,10 @@
         <v>3.12</v>
       </c>
       <c r="J4" s="19" t="n">
-        <v>27.6</v>
+        <v>14.1</v>
       </c>
       <c r="K4" s="31" t="n">
-        <v>35.88</v>
+        <v>18.33</v>
       </c>
     </row>
     <row r="5">
@@ -3860,13 +3860,13 @@
         <v>0.18</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>0.58</v>
+        <v>0.16</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>4.5</v>
+        <v>1.25</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>2.45</v>
+        <v>1.02</v>
       </c>
       <c r="G5" s="26" t="n">
         <v>0</v>
@@ -3878,10 +3878,10 @@
         <v>1.67</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>11.38</v>
+        <v>6.28</v>
       </c>
       <c r="K5" s="32" t="n">
-        <v>14.79</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="6">
@@ -3899,13 +3899,13 @@
         <v>0.28</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>0.29</v>
+        <v>0.01</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>1.15</v>
+        <v>0.48</v>
       </c>
       <c r="G6" s="21" t="n">
         <v>0</v>
@@ -3917,10 +3917,10 @@
         <v>1.67</v>
       </c>
       <c r="J6" s="19" t="n">
-        <v>5.57</v>
+        <v>4.48</v>
       </c>
       <c r="K6" s="31" t="n">
-        <v>7.24</v>
+        <v>5.83</v>
       </c>
     </row>
     <row r="7">
@@ -3938,13 +3938,13 @@
         <v>0.22</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>0.29</v>
+        <v>0.05</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>1.44</v>
+        <v>0.4</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>0.43</v>
+        <v>0.18</v>
       </c>
       <c r="G7" s="26" t="n">
         <v>0</v>
@@ -3956,10 +3956,10 @@
         <v>1.25</v>
       </c>
       <c r="J7" s="24" t="n">
-        <v>5.63</v>
+        <v>4.1</v>
       </c>
       <c r="K7" s="32" t="n">
-        <v>7.32</v>
+        <v>5.34</v>
       </c>
     </row>
     <row r="8">
@@ -3977,13 +3977,13 @@
         <v>0.24</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>0.58</v>
+        <v>0.24</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>6.84</v>
+        <v>1.9</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>0.48</v>
+        <v>0.4</v>
       </c>
       <c r="G8" s="21" t="n">
         <v>0</v>
@@ -3995,10 +3995,10 @@
         <v>3.33</v>
       </c>
       <c r="J8" s="19" t="n">
-        <v>15.46</v>
+        <v>10.11</v>
       </c>
       <c r="K8" s="31" t="n">
-        <v>20.1</v>
+        <v>13.14</v>
       </c>
     </row>
     <row r="9">
@@ -4013,16 +4013,16 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>0.2</v>
+        <v>0.86</v>
       </c>
       <c r="D9" s="26" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="F9" s="26" t="n">
-        <v>0.58</v>
+        <v>1.44</v>
       </c>
       <c r="G9" s="26" t="n">
         <v>0</v>
@@ -4034,10 +4034,10 @@
         <v>1.46</v>
       </c>
       <c r="J9" s="24" t="n">
-        <v>4.24</v>
+        <v>6.24</v>
       </c>
       <c r="K9" s="32" t="n">
-        <v>5.51</v>
+        <v>8.109999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -4052,16 +4052,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>2.31</v>
+        <v>2.96</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>3.17</v>
+        <v>1.01</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>28.8</v>
+        <v>8.48</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>7.1</v>
+        <v>4.36</v>
       </c>
       <c r="G10" s="33" t="n">
         <v>0</v>
@@ -4073,10 +4073,10 @@
         <v>12.5</v>
       </c>
       <c r="J10" s="33" t="n">
-        <v>69.88</v>
+        <v>45.31</v>
       </c>
       <c r="K10" s="33" t="n">
-        <v>90.84</v>
+        <v>58.9</v>
       </c>
     </row>
   </sheetData>
@@ -4180,13 +4180,13 @@
         </is>
       </c>
       <c r="C4" s="21" t="n">
-        <v>1064.1</v>
+        <v>615.9</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>1439</v>
+        <v>972.2</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>6.54</v>
+        <v>4.42</v>
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
@@ -4194,10 +4194,10 @@
         </is>
       </c>
       <c r="G4" s="21" t="n">
-        <v>461.2</v>
+        <v>308</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>1574</v>
+        <v>1051</v>
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
@@ -4222,13 +4222,13 @@
         </is>
       </c>
       <c r="C5" s="26" t="n">
-        <v>453.2</v>
+        <v>282.2</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>790.9</v>
+        <v>610.9</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>3.59</v>
+        <v>2.78</v>
       </c>
       <c r="F5" s="23" t="inlineStr">
         <is>
@@ -4236,10 +4236,10 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>204.8</v>
+        <v>145.1</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>699</v>
+        <v>495</v>
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
@@ -4264,13 +4264,13 @@
         </is>
       </c>
       <c r="C6" s="21" t="n">
-        <v>243.4</v>
+        <v>207</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>565.8</v>
+        <v>527.5</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>2.57</v>
+        <v>2.4</v>
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
@@ -4278,10 +4278,10 @@
         </is>
       </c>
       <c r="G6" s="21" t="n">
-        <v>121.8</v>
+        <v>109.1</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>416</v>
+        <v>372</v>
       </c>
       <c r="I6" s="20" t="inlineStr">
         <is>
@@ -4306,13 +4306,13 @@
         </is>
       </c>
       <c r="C7" s="26" t="n">
-        <v>234</v>
+        <v>182.1</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>555.8</v>
+        <v>500.6</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>2.53</v>
+        <v>2.28</v>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
@@ -4320,10 +4320,10 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>110.9</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>378</v>
+        <v>315</v>
       </c>
       <c r="I7" s="25" t="inlineStr">
         <is>
@@ -4348,13 +4348,13 @@
         </is>
       </c>
       <c r="C8" s="21" t="n">
-        <v>649.5</v>
+        <v>459.2</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>1003.8</v>
+        <v>801.9</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>4.56</v>
+        <v>3.65</v>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
@@ -4362,14 +4362,14 @@
         </is>
       </c>
       <c r="G8" s="21" t="n">
-        <v>311.8</v>
+        <v>238.5</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>1064</v>
+        <v>814</v>
       </c>
       <c r="I8" s="20" t="inlineStr">
         <is>
-          <t>Panel Air Conditioner</t>
+          <t>Fan Filter Unit (IP54)</t>
         </is>
       </c>
       <c r="J8" s="20" t="inlineStr">
@@ -4390,13 +4390,13 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>203.4</v>
+        <v>257.9</v>
       </c>
       <c r="D9" s="26" t="n">
-        <v>526.5</v>
+        <v>580.5</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>2.39</v>
+        <v>2.64</v>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
@@ -4404,10 +4404,10 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>110.8</v>
+        <v>121.8</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>378</v>
+        <v>415</v>
       </c>
       <c r="I9" s="25" t="inlineStr">
         <is>
@@ -5533,17 +5533,17 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>7.45</v>
+        <v>6.12</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>9.69</v>
+        <v>7.96</v>
       </c>
       <c r="F20" s="11" t="n">
         <v>20</v>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>39.8%</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -5552,11 +5552,11 @@
         </is>
       </c>
       <c r="I20" s="11" t="n">
-        <v>17.5</v>
+        <v>14.4</v>
       </c>
       <c r="J20" s="37" t="inlineStr">
         <is>
-          <t>PASS (Optimal Load &lt;50%)</t>
+          <t>PASS (Optimal Load &lt;40%)</t>
         </is>
       </c>
     </row>
@@ -5577,17 +5577,17 @@
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>11.2</v>
+        <v>7.36</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>14.56</v>
+        <v>9.57</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>20</v>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>72.8%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
@@ -5596,11 +5596,11 @@
         </is>
       </c>
       <c r="I21" s="11" t="n">
-        <v>26.2</v>
+        <v>17.3</v>
       </c>
       <c r="J21" s="37" t="inlineStr">
         <is>
-          <t>PASS (Safe Continuous &lt;75%)</t>
+          <t>PASS (Optimal Load &lt;50%)</t>
         </is>
       </c>
     </row>
@@ -5621,17 +5621,17 @@
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>11.38</v>
+        <v>6.11</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>14.79</v>
+        <v>7.94</v>
       </c>
       <c r="F22" s="11" t="n">
         <v>20</v>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -5640,11 +5640,11 @@
         </is>
       </c>
       <c r="I22" s="11" t="n">
-        <v>26.6</v>
+        <v>14.3</v>
       </c>
       <c r="J22" s="37" t="inlineStr">
         <is>
-          <t>PASS (Safe Continuous &lt;75%)</t>
+          <t>PASS (Optimal Load &lt;40%)</t>
         </is>
       </c>
     </row>
@@ -5665,17 +5665,17 @@
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>5.57</v>
+        <v>4.32</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>7.24</v>
+        <v>5.62</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>20</v>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>28.1%</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -5684,11 +5684,11 @@
         </is>
       </c>
       <c r="I23" s="11" t="n">
-        <v>13</v>
+        <v>10.1</v>
       </c>
       <c r="J23" s="37" t="inlineStr">
         <is>
-          <t>PASS (Generous Spare Headroom)</t>
+          <t>PASS (Generous Headroom)</t>
         </is>
       </c>
     </row>
@@ -5709,17 +5709,17 @@
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>5.63</v>
+        <v>4.05</v>
       </c>
       <c r="E24" s="11" t="n">
-        <v>7.32</v>
+        <v>5.27</v>
       </c>
       <c r="F24" s="11" t="n">
         <v>20</v>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>36.6%</t>
+          <t>26.3%</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -5728,11 +5728,11 @@
         </is>
       </c>
       <c r="I24" s="11" t="n">
-        <v>13.2</v>
+        <v>9.5</v>
       </c>
       <c r="J24" s="37" t="inlineStr">
         <is>
-          <t>PASS (Generous Spare Headroom)</t>
+          <t>PASS (Generous Headroom)</t>
         </is>
       </c>
     </row>
@@ -5813,10 +5813,10 @@
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>27.6</v>
+        <v>13.48</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>35.88</v>
+        <v>17.52</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>40</v>
@@ -5828,15 +5828,15 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>89.7% (Single) / 44.9% (Dual)</t>
+          <t>87.6% (Single) / 43.8% (Dual)</t>
         </is>
       </c>
       <c r="I28" s="11" t="n">
-        <v>64</v>
+        <v>31.7</v>
       </c>
       <c r="J28" s="37" t="inlineStr">
         <is>
-          <t>PASS (Sufficient Bus Capacity)</t>
+          <t>PASS (True N+1 Redundancy)</t>
         </is>
       </c>
     </row>
@@ -5857,10 +5857,10 @@
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>11.38</v>
+        <v>6.11</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>14.79</v>
+        <v>7.94</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>20</v>
@@ -5872,15 +5872,15 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>74.0% of nominal 20A</t>
+          <t>39.7% of nominal 20A</t>
         </is>
       </c>
       <c r="I29" s="11" t="n">
-        <v>26.6</v>
+        <v>14.3</v>
       </c>
       <c r="J29" s="37" t="inlineStr">
         <is>
-          <t>PASS (Safe Continuous &lt;75%)</t>
+          <t>PASS (Optimal Load &lt;40%)</t>
         </is>
       </c>
     </row>
@@ -5901,10 +5901,10 @@
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>5.57</v>
+        <v>4.32</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>7.24</v>
+        <v>5.62</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>20</v>
@@ -5916,15 +5916,15 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>36.2% of nominal 20A</t>
+          <t>28.1% of nominal 20A</t>
         </is>
       </c>
       <c r="I30" s="11" t="n">
-        <v>13</v>
+        <v>10.1</v>
       </c>
       <c r="J30" s="37" t="inlineStr">
         <is>
-          <t>PASS (Optimal &lt;50%)</t>
+          <t>PASS (Generous Headroom)</t>
         </is>
       </c>
     </row>
@@ -5945,10 +5945,10 @@
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>5.63</v>
+        <v>4.05</v>
       </c>
       <c r="E31" s="11" t="n">
-        <v>7.32</v>
+        <v>5.27</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>20</v>
@@ -5960,15 +5960,15 @@
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>36.6% of nominal 20A</t>
+          <t>26.3% of nominal 20A</t>
         </is>
       </c>
       <c r="I31" s="11" t="n">
-        <v>13.2</v>
+        <v>9.5</v>
       </c>
       <c r="J31" s="37" t="inlineStr">
         <is>
-          <t>PASS (Optimal &lt;50%)</t>
+          <t>PASS (Generous Headroom)</t>
         </is>
       </c>
     </row>

</xml_diff>